<commit_message>
Add Saudi Arabia Ecommerce and Fashion prospect workbooks; use clean headers in all workbooks
Co-authored-by: abaszeinn-beep <abaszeinn-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/markets/prospects/Kuwait_Ecommerce_Prospects.xlsx
+++ b/markets/prospects/Kuwait_Ecommerce_Prospects.xlsx
@@ -519,12 +519,12 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Company Phone Numbers (comma separated)</t>
+          <t>Company Phone Numbers</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Company Emails (comma separated; marketing/sales/business only)</t>
+          <t>Company Emails</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">

</xml_diff>